<commit_message>
update data files and added two .py
</commit_message>
<xml_diff>
--- a/data/processed/stock analysis 2021-2024 FTSE 100 index.xlsx
+++ b/data/processed/stock analysis 2021-2024 FTSE 100 index.xlsx
@@ -467,19 +467,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7.47</v>
+        <v>6.26</v>
       </c>
       <c r="C2" t="n">
-        <v>747</v>
+        <v>626</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0866</v>
+        <v>-0.1017</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2787</v>
+        <v>0.2361</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.3624</v>
+        <v>-0.4918</v>
       </c>
     </row>
     <row r="3">
@@ -489,19 +489,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.49</v>
+        <v>2.91</v>
       </c>
       <c r="C3" t="n">
-        <v>249</v>
+        <v>291</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0814</v>
+        <v>0.09569999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1847</v>
+        <v>0.167</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3628</v>
+        <v>0.4867</v>
       </c>
     </row>
     <row r="4">
@@ -511,19 +511,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.79</v>
+        <v>4.84</v>
       </c>
       <c r="C4" t="n">
-        <v>379</v>
+        <v>484</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0292</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0543</v>
+        <v>0.097</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2718</v>
+        <v>0.5674</v>
       </c>
     </row>
     <row r="5">
@@ -533,19 +533,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.29</v>
+        <v>5.48</v>
       </c>
       <c r="C5" t="n">
-        <v>429</v>
+        <v>548</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0598</v>
+        <v>0.09429999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>0.09429999999999999</v>
+        <v>0.1002</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4806</v>
+        <v>0.7966</v>
       </c>
     </row>
     <row r="6">
@@ -555,19 +555,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2.61</v>
+        <v>2.49</v>
       </c>
       <c r="C6" t="n">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.0626</v>
+        <v>-0.0587</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1143</v>
+        <v>0.1142</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.674</v>
+        <v>-0.6407</v>
       </c>
     </row>
     <row r="7">
@@ -577,19 +577,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.83</v>
+        <v>1.73</v>
       </c>
       <c r="C7" t="n">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0026</v>
+        <v>-0.0114</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0402</v>
+        <v>0.0379</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.4237</v>
+        <v>-0.6825</v>
       </c>
     </row>
     <row r="8">
@@ -599,19 +599,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2.49</v>
+        <v>2.47</v>
       </c>
       <c r="C8" t="n">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0415</v>
+        <v>-0.0359</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1047</v>
+        <v>0.09470000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.5342</v>
+        <v>-0.5321</v>
       </c>
     </row>
     <row r="9">
@@ -621,19 +621,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.655</v>
       </c>
       <c r="C9" t="n">
-        <v>56</v>
+        <v>65.5</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0371</v>
+        <v>0.0601</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3029</v>
+        <v>0.2806</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0747</v>
+        <v>0.1626</v>
       </c>
     </row>
     <row r="10">
@@ -643,19 +643,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8.84</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="C10" t="n">
-        <v>884</v>
+        <v>896</v>
       </c>
       <c r="D10" t="n">
-        <v>0.07340000000000001</v>
+        <v>0.0667</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0732</v>
+        <v>0.1176</v>
       </c>
       <c r="F10" t="n">
-        <v>0.8053</v>
+        <v>0.4445</v>
       </c>
     </row>
     <row r="11">
@@ -665,19 +665,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>18.7</v>
+        <v>20.66</v>
       </c>
       <c r="C11" t="n">
-        <v>1870</v>
+        <v>2066</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.0117</v>
+        <v>0.0077</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0926</v>
+        <v>0.0949</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.2825</v>
+        <v>-0.07149999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -687,19 +687,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3.68</v>
+        <v>3.62</v>
       </c>
       <c r="C12" t="n">
-        <v>368</v>
+        <v>362</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.0015</v>
+        <v>-0.0045</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1112</v>
+        <v>0.09470000000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1437</v>
+        <v>-0.1997</v>
       </c>
     </row>
     <row r="13">
@@ -709,19 +709,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3.48</v>
+        <v>2.38</v>
       </c>
       <c r="C13" t="n">
-        <v>348</v>
+        <v>238</v>
       </c>
       <c r="D13" t="n">
-        <v>0.136</v>
+        <v>0.0578</v>
       </c>
       <c r="E13" t="n">
-        <v>0.4881</v>
+        <v>0.4695</v>
       </c>
       <c r="F13" t="n">
-        <v>0.249</v>
+        <v>0.0924</v>
       </c>
     </row>
     <row r="14">
@@ -731,19 +731,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6.8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C14" t="n">
-        <v>680</v>
+        <v>820</v>
       </c>
       <c r="D14" t="n">
-        <v>0.057</v>
+        <v>0.08160000000000001</v>
       </c>
       <c r="E14" t="n">
-        <v>0.06909999999999999</v>
+        <v>0.0835</v>
       </c>
       <c r="F14" t="n">
-        <v>0.615</v>
+        <v>0.8041</v>
       </c>
     </row>
     <row r="15">
@@ -753,19 +753,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1.48</v>
+        <v>1.2</v>
       </c>
       <c r="C15" t="n">
-        <v>148</v>
+        <v>120</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0225</v>
+        <v>-0.0517</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0935</v>
+        <v>0.09279999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.3955</v>
+        <v>-0.7127</v>
       </c>
     </row>
     <row r="16">
@@ -775,19 +775,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.63</v>
+        <v>2.09</v>
       </c>
       <c r="C16" t="n">
-        <v>263</v>
+        <v>209</v>
       </c>
       <c r="D16" t="n">
-        <v>0.2541</v>
+        <v>0.1852</v>
       </c>
       <c r="E16" t="n">
-        <v>0.2301</v>
+        <v>0.3073</v>
       </c>
       <c r="F16" t="n">
-        <v>1.0416</v>
+        <v>0.5556</v>
       </c>
     </row>
     <row r="17">
@@ -797,19 +797,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2.39</v>
+        <v>1.85</v>
       </c>
       <c r="C17" t="n">
-        <v>239</v>
+        <v>185</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0052</v>
+        <v>-0.0273</v>
       </c>
       <c r="E17" t="n">
-        <v>0.2227</v>
+        <v>0.2549</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0415</v>
+        <v>-0.1637</v>
       </c>
     </row>
     <row r="18">
@@ -819,19 +819,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.64</v>
+        <v>0.515</v>
       </c>
       <c r="C18" t="n">
-        <v>64</v>
+        <v>51.5</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0076</v>
+        <v>-0.0513</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0155</v>
+        <v>0.1287</v>
       </c>
       <c r="F18" t="n">
-        <v>-1.4253</v>
+        <v>-0.5105</v>
       </c>
     </row>
     <row r="19">
@@ -841,19 +841,19 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1.5</v>
+        <v>2.09</v>
       </c>
       <c r="C19" t="n">
-        <v>150</v>
+        <v>209</v>
       </c>
       <c r="D19" t="n">
-        <v>0.1352</v>
+        <v>0.1769</v>
       </c>
       <c r="E19" t="n">
-        <v>0.2862</v>
+        <v>0.2689</v>
       </c>
       <c r="F19" t="n">
-        <v>0.4219</v>
+        <v>0.604</v>
       </c>
     </row>
     <row r="20">
@@ -863,19 +863,19 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1.52</v>
+        <v>1.86</v>
       </c>
       <c r="C20" t="n">
-        <v>152</v>
+        <v>186</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.0068</v>
+        <v>0.0342</v>
       </c>
       <c r="E20" t="n">
-        <v>0.1413</v>
+        <v>0.1815</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.1507</v>
+        <v>0.1089</v>
       </c>
     </row>
     <row r="21">
@@ -885,19 +885,19 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>31.78</v>
+        <v>28.18</v>
       </c>
       <c r="C21" t="n">
-        <v>3178</v>
+        <v>2818</v>
       </c>
       <c r="D21" t="n">
-        <v>0.057</v>
+        <v>0.0274</v>
       </c>
       <c r="E21" t="n">
-        <v>0.1144</v>
+        <v>0.112</v>
       </c>
       <c r="F21" t="n">
-        <v>0.3715</v>
+        <v>0.116</v>
       </c>
     </row>
     <row r="22">
@@ -913,13 +913,13 @@
         <v>446</v>
       </c>
       <c r="D22" t="n">
-        <v>0.0774</v>
+        <v>0.063</v>
       </c>
       <c r="E22" t="n">
-        <v>0.1484</v>
+        <v>0.1192</v>
       </c>
       <c r="F22" t="n">
-        <v>0.424</v>
+        <v>0.4071</v>
       </c>
     </row>
     <row r="23">
@@ -929,19 +929,19 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6.58</v>
+        <v>4.74</v>
       </c>
       <c r="C23" t="n">
-        <v>658</v>
+        <v>474</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1947</v>
+        <v>0.1383</v>
       </c>
       <c r="E23" t="n">
-        <v>0.1316</v>
+        <v>0.3223</v>
       </c>
       <c r="F23" t="n">
-        <v>1.3693</v>
+        <v>0.3844</v>
       </c>
     </row>
     <row r="24">
@@ -951,19 +951,19 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3.6</v>
+        <v>4.29</v>
       </c>
       <c r="C24" t="n">
-        <v>360</v>
+        <v>429</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0658</v>
+        <v>0.08690000000000001</v>
       </c>
       <c r="E24" t="n">
-        <v>0.1149</v>
+        <v>0.1167</v>
       </c>
       <c r="F24" t="n">
-        <v>0.447</v>
+        <v>0.6213</v>
       </c>
     </row>
     <row r="25">
@@ -973,19 +973,19 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4.71</v>
+        <v>3.86</v>
       </c>
       <c r="C25" t="n">
-        <v>471</v>
+        <v>386</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0185</v>
+        <v>-0.0145</v>
       </c>
       <c r="E25" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.116</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0449</v>
+        <v>-0.2496</v>
       </c>
     </row>
     <row r="26">
@@ -995,19 +995,19 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2.55</v>
+        <v>2.26</v>
       </c>
       <c r="C26" t="n">
-        <v>255</v>
+        <v>226</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.0119</v>
+        <v>-0.0286</v>
       </c>
       <c r="E26" t="n">
-        <v>0.0644</v>
+        <v>0.0745</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.4087</v>
+        <v>-0.5776</v>
       </c>
     </row>
     <row r="27">
@@ -1017,19 +1017,19 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="C27" t="n">
-        <v>600</v>
+        <v>590</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.0132</v>
+        <v>-0.013</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0447</v>
+        <v>0.0579</v>
       </c>
       <c r="F27" t="n">
-        <v>-0.6189</v>
+        <v>-0.4743</v>
       </c>
     </row>
     <row r="28">
@@ -1039,19 +1039,19 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>5.25</v>
+        <v>2.31</v>
       </c>
       <c r="C28" t="n">
-        <v>525</v>
+        <v>231</v>
       </c>
       <c r="D28" t="n">
-        <v>0.0204</v>
+        <v>-0.075</v>
       </c>
       <c r="E28" t="n">
-        <v>0.2183</v>
+        <v>0.3106</v>
       </c>
       <c r="F28" t="n">
-        <v>0.0272</v>
+        <v>-0.288</v>
       </c>
     </row>
     <row r="29">
@@ -1061,19 +1061,19 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>3.68</v>
+        <v>3.95</v>
       </c>
       <c r="C29" t="n">
-        <v>368</v>
+        <v>395</v>
       </c>
       <c r="D29" t="n">
-        <v>0.1628</v>
+        <v>0.156</v>
       </c>
       <c r="E29" t="n">
-        <v>0.6074000000000001</v>
+        <v>0.5816</v>
       </c>
       <c r="F29" t="n">
-        <v>0.2443</v>
+        <v>0.2433</v>
       </c>
     </row>
     <row r="30">
@@ -1083,19 +1083,19 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>3.28</v>
+        <v>3.95</v>
       </c>
       <c r="C30" t="n">
-        <v>328</v>
+        <v>395</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0275</v>
+        <v>0.0123</v>
       </c>
       <c r="E30" t="n">
-        <v>0.4138</v>
+        <v>0.387</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1013</v>
+        <v>-0.0056</v>
       </c>
     </row>
     <row r="31">
@@ -1105,19 +1105,19 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>22.04</v>
+        <v>24.12</v>
       </c>
       <c r="C31" t="n">
-        <v>2204</v>
+        <v>2412</v>
       </c>
       <c r="D31" t="n">
-        <v>0.0226</v>
+        <v>0.0336</v>
       </c>
       <c r="E31" t="n">
-        <v>0.143</v>
+        <v>0.1221</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0571</v>
+        <v>0.1567</v>
       </c>
     </row>
     <row r="32">
@@ -1127,19 +1127,19 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.865</v>
+        <v>0.885</v>
       </c>
       <c r="C32" t="n">
-        <v>86.5</v>
+        <v>88.5</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.0292</v>
+        <v>-0.0207</v>
       </c>
       <c r="E32" t="n">
-        <v>0.393</v>
+        <v>0.3513</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.1111</v>
+        <v>-0.1002</v>
       </c>
     </row>
     <row r="33">
@@ -1149,19 +1149,19 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>19.2</v>
+        <v>20.56</v>
       </c>
       <c r="C33" t="n">
-        <v>1920</v>
+        <v>2056</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.0011</v>
+        <v>0.0108</v>
       </c>
       <c r="E33" t="n">
-        <v>0.0489</v>
+        <v>0.0516</v>
       </c>
       <c r="F33" t="n">
-        <v>-0.3184</v>
+        <v>-0.07049999999999999</v>
       </c>
     </row>
     <row r="34">
@@ -1171,19 +1171,19 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1.84</v>
+        <v>2.14</v>
       </c>
       <c r="C34" t="n">
-        <v>184</v>
+        <v>214</v>
       </c>
       <c r="D34" t="n">
-        <v>0.0374</v>
+        <v>0.0579</v>
       </c>
       <c r="E34" t="n">
-        <v>0.055</v>
+        <v>0.0605</v>
       </c>
       <c r="F34" t="n">
-        <v>0.4186</v>
+        <v>0.7184</v>
       </c>
     </row>
     <row r="35">
@@ -1193,19 +1193,19 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>6.3</v>
+        <v>7.3</v>
       </c>
       <c r="C35" t="n">
-        <v>630</v>
+        <v>730</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.004</v>
+        <v>0.0232</v>
       </c>
       <c r="E35" t="n">
-        <v>0.0423</v>
+        <v>0.0764</v>
       </c>
       <c r="F35" t="n">
-        <v>-0.4352</v>
+        <v>0.114</v>
       </c>
     </row>
     <row r="36">
@@ -1215,19 +1215,19 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3.05</v>
+        <v>3.04</v>
       </c>
       <c r="C36" t="n">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D36" t="n">
-        <v>0.1869</v>
+        <v>0.1673</v>
       </c>
       <c r="E36" t="n">
-        <v>0.2484</v>
+        <v>0.3021</v>
       </c>
       <c r="F36" t="n">
-        <v>0.6942</v>
+        <v>0.5059</v>
       </c>
     </row>
     <row r="37">
@@ -1237,19 +1237,19 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3.7</v>
+        <v>3.06</v>
       </c>
       <c r="C37" t="n">
-        <v>370</v>
+        <v>306</v>
       </c>
       <c r="D37" t="n">
-        <v>0.031</v>
+        <v>-0.0018</v>
       </c>
       <c r="E37" t="n">
-        <v>0.1405</v>
+        <v>0.1606</v>
       </c>
       <c r="F37" t="n">
-        <v>0.1175</v>
+        <v>-0.1009</v>
       </c>
     </row>
     <row r="38">
@@ -1259,19 +1259,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3.7</v>
+        <v>3.88</v>
       </c>
       <c r="C38" t="n">
-        <v>370</v>
+        <v>388</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.0026</v>
+        <v>0.0055</v>
       </c>
       <c r="E38" t="n">
-        <v>0.0746</v>
+        <v>0.0614</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2287</v>
+        <v>-0.1462</v>
       </c>
     </row>
     <row r="39">
@@ -1281,19 +1281,19 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2.21</v>
+        <v>2.24</v>
       </c>
       <c r="C39" t="n">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D39" t="n">
-        <v>0.1853</v>
+        <v>0.1568</v>
       </c>
       <c r="E39" t="n">
-        <v>0.2416</v>
+        <v>0.228</v>
       </c>
       <c r="F39" t="n">
-        <v>0.707</v>
+        <v>0.6245000000000001</v>
       </c>
     </row>
     <row r="40">
@@ -1303,19 +1303,19 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2.56</v>
+        <v>3.69</v>
       </c>
       <c r="C40" t="n">
-        <v>256</v>
+        <v>369</v>
       </c>
       <c r="D40" t="n">
-        <v>0.2316</v>
+        <v>0.284</v>
       </c>
       <c r="E40" t="n">
-        <v>0.2258</v>
+        <v>0.2122</v>
       </c>
       <c r="F40" t="n">
-        <v>0.9614</v>
+        <v>1.2706</v>
       </c>
     </row>
     <row r="41">
@@ -1325,19 +1325,19 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1.81</v>
+        <v>2.21</v>
       </c>
       <c r="C41" t="n">
-        <v>181</v>
+        <v>221</v>
       </c>
       <c r="D41" t="n">
-        <v>0.1204</v>
+        <v>0.1364</v>
       </c>
       <c r="E41" t="n">
-        <v>0.2381</v>
+        <v>0.2122</v>
       </c>
       <c r="F41" t="n">
-        <v>0.4449</v>
+        <v>0.5747</v>
       </c>
     </row>
     <row r="42">
@@ -1347,19 +1347,19 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2.35</v>
+        <v>2.83</v>
       </c>
       <c r="C42" t="n">
-        <v>235</v>
+        <v>283</v>
       </c>
       <c r="D42" t="n">
-        <v>0.0953</v>
+        <v>0.1165</v>
       </c>
       <c r="E42" t="n">
-        <v>0.3217</v>
+        <v>0.3065</v>
       </c>
       <c r="F42" t="n">
-        <v>0.2512</v>
+        <v>0.3329</v>
       </c>
     </row>
     <row r="43">
@@ -1369,19 +1369,19 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1.93</v>
+        <v>2.43</v>
       </c>
       <c r="C43" t="n">
-        <v>193</v>
+        <v>243</v>
       </c>
       <c r="D43" t="n">
-        <v>0.1471</v>
+        <v>0.1664</v>
       </c>
       <c r="E43" t="n">
-        <v>0.2033</v>
+        <v>0.1928</v>
       </c>
       <c r="F43" t="n">
-        <v>0.6526</v>
+        <v>0.7883</v>
       </c>
     </row>
     <row r="44">
@@ -1391,19 +1391,19 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>20.64</v>
+        <v>21.8</v>
       </c>
       <c r="C44" t="n">
-        <v>2064</v>
+        <v>2180</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.0075</v>
+        <v>0.0027</v>
       </c>
       <c r="E44" t="n">
-        <v>0.0625</v>
+        <v>0.054</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.3516</v>
+        <v>-0.2169</v>
       </c>
     </row>
     <row r="45">
@@ -1413,19 +1413,19 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1.73</v>
+        <v>1.8</v>
       </c>
       <c r="C45" t="n">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="D45" t="n">
-        <v>0.2498</v>
+        <v>0.2277</v>
       </c>
       <c r="E45" t="n">
-        <v>0.3816</v>
+        <v>0.4193</v>
       </c>
       <c r="F45" t="n">
-        <v>0.6168</v>
+        <v>0.5086000000000001</v>
       </c>
     </row>
     <row r="46">
@@ -1435,19 +1435,19 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.765</v>
+        <v>0.845</v>
       </c>
       <c r="C46" t="n">
-        <v>76.5</v>
+        <v>84.5</v>
       </c>
       <c r="D46" t="n">
-        <v>0.0131</v>
+        <v>0.0306</v>
       </c>
       <c r="E46" t="n">
-        <v>0.0982</v>
+        <v>0.1257</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.0133</v>
+        <v>0.1287</v>
       </c>
     </row>
     <row r="47">
@@ -1457,19 +1457,19 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>9.960000000000001</v>
+        <v>10.24</v>
       </c>
       <c r="C47" t="n">
-        <v>996</v>
+        <v>1024</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0384</v>
+        <v>0.037</v>
       </c>
       <c r="E47" t="n">
-        <v>0.0366</v>
+        <v>0.0437</v>
       </c>
       <c r="F47" t="n">
-        <v>0.6554</v>
+        <v>0.5165999999999999</v>
       </c>
     </row>
     <row r="48">
@@ -1479,19 +1479,19 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>4.98</v>
+        <v>4.9</v>
       </c>
       <c r="C48" t="n">
-        <v>498</v>
+        <v>490</v>
       </c>
       <c r="D48" t="n">
-        <v>0.1956</v>
+        <v>0.1655</v>
       </c>
       <c r="E48" t="n">
-        <v>0.1962</v>
+        <v>0.2222</v>
       </c>
       <c r="F48" t="n">
-        <v>0.9231</v>
+        <v>0.6798999999999999</v>
       </c>
     </row>
     <row r="49">
@@ -1501,19 +1501,19 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>39.42</v>
+        <v>25.9</v>
       </c>
       <c r="C49" t="n">
-        <v>3942</v>
+        <v>2590</v>
       </c>
       <c r="D49" t="n">
-        <v>0.0221</v>
+        <v>-0.0447</v>
       </c>
       <c r="E49" t="n">
-        <v>0.2563</v>
+        <v>0.2419</v>
       </c>
       <c r="F49" t="n">
-        <v>0.0298</v>
+        <v>-0.2445</v>
       </c>
     </row>
     <row r="50">
@@ -1523,19 +1523,19 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.605</v>
+        <v>0.525</v>
       </c>
       <c r="C50" t="n">
-        <v>60.5</v>
+        <v>52.5</v>
       </c>
       <c r="D50" t="n">
-        <v>0.1528</v>
+        <v>0.1056</v>
       </c>
       <c r="E50" t="n">
-        <v>0.3232</v>
+        <v>0.3126</v>
       </c>
       <c r="F50" t="n">
-        <v>0.428</v>
+        <v>0.2918</v>
       </c>
     </row>
     <row r="51">
@@ -1545,19 +1545,19 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1.78</v>
+        <v>2.39</v>
       </c>
       <c r="C51" t="n">
-        <v>178</v>
+        <v>239</v>
       </c>
       <c r="D51" t="n">
-        <v>-0.0277</v>
+        <v>0.0313</v>
       </c>
       <c r="E51" t="n">
-        <v>0.1998</v>
+        <v>0.2146</v>
       </c>
       <c r="F51" t="n">
-        <v>-0.2108</v>
+        <v>0.0785</v>
       </c>
     </row>
     <row r="52">
@@ -1567,19 +1567,19 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>3.53</v>
+        <v>3.65</v>
       </c>
       <c r="C52" t="n">
-        <v>353</v>
+        <v>365</v>
       </c>
       <c r="D52" t="n">
-        <v>-0.0327</v>
+        <v>-0.0216</v>
       </c>
       <c r="E52" t="n">
-        <v>0.0828</v>
+        <v>0.0789</v>
       </c>
       <c r="F52" t="n">
-        <v>-0.5699</v>
+        <v>-0.457</v>
       </c>
     </row>
     <row r="53">
@@ -1589,19 +1589,19 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.74</v>
       </c>
       <c r="C53" t="n">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="D53" t="n">
-        <v>0.0789</v>
+        <v>0.0515</v>
       </c>
       <c r="E53" t="n">
-        <v>0.1309</v>
+        <v>0.1368</v>
       </c>
       <c r="F53" t="n">
-        <v>0.4922</v>
+        <v>0.2709</v>
       </c>
     </row>
     <row r="54">
@@ -1611,19 +1611,19 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>4.71</v>
+        <v>4.59</v>
       </c>
       <c r="C54" t="n">
-        <v>471</v>
+        <v>459</v>
       </c>
       <c r="D54" t="n">
-        <v>0.065</v>
+        <v>0.0511</v>
       </c>
       <c r="E54" t="n">
-        <v>0.1226</v>
+        <v>0.1288</v>
       </c>
       <c r="F54" t="n">
-        <v>0.4123</v>
+        <v>0.2845</v>
       </c>
     </row>
     <row r="55">
@@ -1633,19 +1633,19 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>8.52</v>
+        <v>7.6</v>
       </c>
       <c r="C55" t="n">
-        <v>852</v>
+        <v>760</v>
       </c>
       <c r="D55" t="n">
-        <v>0.043</v>
+        <v>0.0194</v>
       </c>
       <c r="E55" t="n">
-        <v>0.0677</v>
+        <v>0.1065</v>
       </c>
       <c r="F55" t="n">
-        <v>0.4209</v>
+        <v>0.0462</v>
       </c>
     </row>
     <row r="56">
@@ -1655,19 +1655,19 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1.94</v>
+        <v>1.85</v>
       </c>
       <c r="C56" t="n">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="D56" t="n">
-        <v>-0.0801</v>
+        <v>-0.0673</v>
       </c>
       <c r="E56" t="n">
-        <v>0.2953</v>
+        <v>0.3083</v>
       </c>
       <c r="F56" t="n">
-        <v>-0.3202</v>
+        <v>-0.265</v>
       </c>
     </row>
     <row r="57">
@@ -1677,19 +1677,19 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1.83</v>
+        <v>2.53</v>
       </c>
       <c r="C57" t="n">
-        <v>183</v>
+        <v>253</v>
       </c>
       <c r="D57" t="n">
-        <v>0.1892</v>
+        <v>0.2427</v>
       </c>
       <c r="E57" t="n">
-        <v>0.2645</v>
+        <v>0.277</v>
       </c>
       <c r="F57" t="n">
-        <v>0.6606</v>
+        <v>0.8241000000000001</v>
       </c>
     </row>
     <row r="58">
@@ -1699,19 +1699,19 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>121.5</v>
+        <v>99.98</v>
       </c>
       <c r="C58" t="n">
-        <v>12150</v>
+        <v>9998</v>
       </c>
       <c r="D58" t="n">
-        <v>-0.0153</v>
+        <v>-0.0439</v>
       </c>
       <c r="E58" t="n">
-        <v>0.0529</v>
+        <v>0.055</v>
       </c>
       <c r="F58" t="n">
-        <v>-0.5610000000000001</v>
+        <v>-1.0612</v>
       </c>
     </row>
     <row r="59">
@@ -1721,19 +1721,19 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>6.79</v>
+        <v>7.22</v>
       </c>
       <c r="C59" t="n">
-        <v>679</v>
+        <v>722</v>
       </c>
       <c r="D59" t="n">
-        <v>0.0519</v>
+        <v>0.0539</v>
       </c>
       <c r="E59" t="n">
-        <v>0.1129</v>
+        <v>0.1016</v>
       </c>
       <c r="F59" t="n">
-        <v>0.3319</v>
+        <v>0.3879</v>
       </c>
     </row>
     <row r="60">
@@ -1743,19 +1743,19 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1.59</v>
+        <v>1.78</v>
       </c>
       <c r="C60" t="n">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="D60" t="n">
-        <v>0.137</v>
+        <v>0.1342</v>
       </c>
       <c r="E60" t="n">
-        <v>0.1394</v>
+        <v>0.1258</v>
       </c>
       <c r="F60" t="n">
-        <v>0.8792</v>
+        <v>0.9522</v>
       </c>
     </row>
     <row r="61">
@@ -1765,19 +1765,19 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1.39</v>
+        <v>1.55</v>
       </c>
       <c r="C61" t="n">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="D61" t="n">
-        <v>0.0221</v>
+        <v>0.0381</v>
       </c>
       <c r="E61" t="n">
-        <v>0.0746</v>
+        <v>0.0857</v>
       </c>
       <c r="F61" t="n">
-        <v>0.1026</v>
+        <v>0.2764</v>
       </c>
     </row>
     <row r="62">
@@ -1787,19 +1787,19 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>5.02</v>
+        <v>4.16</v>
       </c>
       <c r="C62" t="n">
-        <v>502</v>
+        <v>416</v>
       </c>
       <c r="D62" t="n">
-        <v>0.0586</v>
+        <v>0.0186</v>
       </c>
       <c r="E62" t="n">
-        <v>0.2001</v>
+        <v>0.1913</v>
       </c>
       <c r="F62" t="n">
-        <v>0.2205</v>
+        <v>0.0215</v>
       </c>
     </row>
     <row r="63">
@@ -1809,19 +1809,19 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>6.31</v>
+        <v>5.17</v>
       </c>
       <c r="C63" t="n">
-        <v>631</v>
+        <v>517</v>
       </c>
       <c r="D63" t="n">
-        <v>-0.0645</v>
+        <v>-0.0844</v>
       </c>
       <c r="E63" t="n">
-        <v>0.0636</v>
+        <v>0.0663</v>
       </c>
       <c r="F63" t="n">
-        <v>-1.2405</v>
+        <v>-1.4914</v>
       </c>
     </row>
     <row r="64">
@@ -1831,19 +1831,19 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>17.44</v>
+        <v>19.32</v>
       </c>
       <c r="C64" t="n">
-        <v>1744</v>
+        <v>1932</v>
       </c>
       <c r="D64" t="n">
-        <v>-0.0144</v>
+        <v>0.0051</v>
       </c>
       <c r="E64" t="n">
-        <v>0.1273</v>
+        <v>0.1172</v>
       </c>
       <c r="F64" t="n">
-        <v>-0.227</v>
+        <v>-0.0794</v>
       </c>
     </row>
     <row r="65">
@@ -1853,19 +1853,19 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>17.82</v>
+        <v>17.68</v>
       </c>
       <c r="C65" t="n">
-        <v>1782</v>
+        <v>1768</v>
       </c>
       <c r="D65" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.007</v>
       </c>
       <c r="E65" t="n">
-        <v>0.0206</v>
+        <v>0.0259</v>
       </c>
       <c r="F65" t="n">
-        <v>-0.2217</v>
+        <v>-0.2858</v>
       </c>
     </row>
     <row r="66">
@@ -1875,19 +1875,19 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>14.3</v>
+        <v>12.4</v>
       </c>
       <c r="C66" t="n">
-        <v>1430</v>
+        <v>1240</v>
       </c>
       <c r="D66" t="n">
-        <v>-0.018</v>
+        <v>-0.0362</v>
       </c>
       <c r="E66" t="n">
-        <v>0.08110000000000001</v>
+        <v>0.09719999999999999</v>
       </c>
       <c r="F66" t="n">
-        <v>-0.4002</v>
+        <v>-0.5215</v>
       </c>
     </row>
     <row r="67">
@@ -1897,19 +1897,19 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>5.76</v>
+        <v>4.9</v>
       </c>
       <c r="C67" t="n">
-        <v>576</v>
+        <v>490</v>
       </c>
       <c r="D67" t="n">
-        <v>-0.0033</v>
+        <v>-0.0311</v>
       </c>
       <c r="E67" t="n">
-        <v>0.1576</v>
+        <v>0.1198</v>
       </c>
       <c r="F67" t="n">
-        <v>-0.1126</v>
+        <v>-0.3803</v>
       </c>
     </row>
     <row r="68">
@@ -1919,19 +1919,19 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>4.02</v>
+        <v>4.56</v>
       </c>
       <c r="C68" t="n">
-        <v>402</v>
+        <v>456</v>
       </c>
       <c r="D68" t="n">
-        <v>-0.0064</v>
+        <v>0.0157</v>
       </c>
       <c r="E68" t="n">
-        <v>0.0834</v>
+        <v>0.07489999999999999</v>
       </c>
       <c r="F68" t="n">
-        <v>-0.2502</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="69">
@@ -1941,19 +1941,19 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>6.52</v>
+        <v>4.76</v>
       </c>
       <c r="C69" t="n">
-        <v>652</v>
+        <v>476</v>
       </c>
       <c r="D69" t="n">
-        <v>0.0579</v>
+        <v>0.005</v>
       </c>
       <c r="E69" t="n">
-        <v>0.0736</v>
+        <v>0.1601</v>
       </c>
       <c r="F69" t="n">
-        <v>0.5908</v>
+        <v>-0.0593</v>
       </c>
     </row>
     <row r="70">
@@ -1963,19 +1963,19 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>2.82</v>
+        <v>1.55</v>
       </c>
       <c r="C70" t="n">
-        <v>282</v>
+        <v>155</v>
       </c>
       <c r="D70" t="n">
-        <v>0.1138</v>
+        <v>0.0245</v>
       </c>
       <c r="E70" t="n">
-        <v>0.2145</v>
+        <v>0.3077</v>
       </c>
       <c r="F70" t="n">
-        <v>0.4633</v>
+        <v>0.0326</v>
       </c>
     </row>
     <row r="71">
@@ -1985,19 +1985,19 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>5.51</v>
+        <v>6.48</v>
       </c>
       <c r="C71" t="n">
-        <v>551</v>
+        <v>648</v>
       </c>
       <c r="D71" t="n">
-        <v>-0.0014</v>
+        <v>0.0273</v>
       </c>
       <c r="E71" t="n">
-        <v>0.0332</v>
+        <v>0.0604</v>
       </c>
       <c r="F71" t="n">
-        <v>-0.4765</v>
+        <v>0.2124</v>
       </c>
     </row>
     <row r="72">
@@ -2007,19 +2007,19 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1.38</v>
+        <v>1.46</v>
       </c>
       <c r="C72" t="n">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="D72" t="n">
-        <v>0.0805</v>
+        <v>0.09329999999999999</v>
       </c>
       <c r="E72" t="n">
-        <v>0.3873</v>
+        <v>0.4262</v>
       </c>
       <c r="F72" t="n">
-        <v>0.1707</v>
+        <v>0.185</v>
       </c>
     </row>
     <row r="73">
@@ -2029,19 +2029,19 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>6.15</v>
+        <v>4.36</v>
       </c>
       <c r="C73" t="n">
-        <v>615</v>
+        <v>436</v>
       </c>
       <c r="D73" t="n">
-        <v>-0.0126</v>
+        <v>-0.0709</v>
       </c>
       <c r="E73" t="n">
-        <v>0.5919</v>
+        <v>0.5012</v>
       </c>
       <c r="F73" t="n">
-        <v>-0.0457</v>
+        <v>-0.1702</v>
       </c>
     </row>
     <row r="74">
@@ -2051,19 +2051,19 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>2.82</v>
+        <v>3.18</v>
       </c>
       <c r="C74" t="n">
-        <v>282</v>
+        <v>318</v>
       </c>
       <c r="D74" t="n">
-        <v>-0.0479</v>
+        <v>-0.019</v>
       </c>
       <c r="E74" t="n">
-        <v>0.1263</v>
+        <v>0.1307</v>
       </c>
       <c r="F74" t="n">
-        <v>-0.4941</v>
+        <v>-0.2557</v>
       </c>
     </row>
     <row r="75">
@@ -2073,19 +2073,19 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>4.31</v>
+        <v>4.44</v>
       </c>
       <c r="C75" t="n">
-        <v>431</v>
+        <v>444</v>
       </c>
       <c r="D75" t="n">
-        <v>-0.0028</v>
+        <v>0.0026</v>
       </c>
       <c r="E75" t="n">
-        <v>0.1467</v>
+        <v>0.131</v>
       </c>
       <c r="F75" t="n">
-        <v>-0.1176</v>
+        <v>-0.09030000000000001</v>
       </c>
     </row>
     <row r="76">
@@ -2095,19 +2095,19 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>4.22</v>
+        <v>4.95</v>
       </c>
       <c r="C76" t="n">
-        <v>422</v>
+        <v>495</v>
       </c>
       <c r="D76" t="n">
-        <v>0.041</v>
+        <v>0.0615</v>
       </c>
       <c r="E76" t="n">
-        <v>0.1144</v>
+        <v>0.09760000000000001</v>
       </c>
       <c r="F76" t="n">
-        <v>0.2325</v>
+        <v>0.4822</v>
       </c>
     </row>
     <row r="77">
@@ -2117,19 +2117,19 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>2.62</v>
+        <v>2.36</v>
       </c>
       <c r="C77" t="n">
-        <v>262</v>
+        <v>236</v>
       </c>
       <c r="D77" t="n">
-        <v>0.0424</v>
+        <v>0.0186</v>
       </c>
       <c r="E77" t="n">
-        <v>0.0732</v>
+        <v>0.0844</v>
       </c>
       <c r="F77" t="n">
-        <v>0.3825</v>
+        <v>0.0492</v>
       </c>
     </row>
     <row r="78">
@@ -2139,19 +2139,19 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>1.34</v>
+        <v>1.69</v>
       </c>
       <c r="C78" t="n">
-        <v>134</v>
+        <v>169</v>
       </c>
       <c r="D78" t="n">
-        <v>0.2201</v>
+        <v>0.2469</v>
       </c>
       <c r="E78" t="n">
-        <v>0.3437</v>
+        <v>0.4271</v>
       </c>
       <c r="F78" t="n">
-        <v>0.5984</v>
+        <v>0.5444</v>
       </c>
     </row>
     <row r="79">
@@ -2161,19 +2161,19 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>3.61</v>
+        <v>4.79</v>
       </c>
       <c r="C79" t="n">
-        <v>361</v>
+        <v>479</v>
       </c>
       <c r="D79" t="n">
-        <v>0.1793</v>
+        <v>0.2112</v>
       </c>
       <c r="E79" t="n">
-        <v>0.2351</v>
+        <v>0.2715</v>
       </c>
       <c r="F79" t="n">
-        <v>0.7013</v>
+        <v>0.7246</v>
       </c>
     </row>
     <row r="80">
@@ -2183,19 +2183,19 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>3.79</v>
+        <v>4.63</v>
       </c>
       <c r="C80" t="n">
-        <v>379</v>
+        <v>463</v>
       </c>
       <c r="D80" t="n">
-        <v>0.2319</v>
+        <v>0.2622</v>
       </c>
       <c r="E80" t="n">
-        <v>0.265</v>
+        <v>0.437</v>
       </c>
       <c r="F80" t="n">
-        <v>0.8206</v>
+        <v>0.5669</v>
       </c>
     </row>
     <row r="81">
@@ -2205,19 +2205,19 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>1.55</v>
+        <v>1.85</v>
       </c>
       <c r="C81" t="n">
-        <v>155</v>
+        <v>185</v>
       </c>
       <c r="D81" t="n">
-        <v>0.023</v>
+        <v>0.0502</v>
       </c>
       <c r="E81" t="n">
-        <v>0.0509</v>
+        <v>0.0605</v>
       </c>
       <c r="F81" t="n">
-        <v>0.1691</v>
+        <v>0.592</v>
       </c>
     </row>
     <row r="82">
@@ -2227,19 +2227,19 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>3.73</v>
+        <v>3.89</v>
       </c>
       <c r="C82" t="n">
-        <v>373</v>
+        <v>389</v>
       </c>
       <c r="D82" t="n">
-        <v>0.0069</v>
+        <v>0.0129</v>
       </c>
       <c r="E82" t="n">
-        <v>0.0708</v>
+        <v>0.065</v>
       </c>
       <c r="F82" t="n">
-        <v>-0.107</v>
+        <v>-0.0242</v>
       </c>
     </row>
     <row r="83">
@@ -2249,19 +2249,19 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>1.08</v>
+        <v>1.98</v>
       </c>
       <c r="C83" t="n">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="D83" t="n">
-        <v>0.4849</v>
+        <v>0.5412</v>
       </c>
       <c r="E83" t="n">
-        <v>0.4464</v>
+        <v>0.411</v>
       </c>
       <c r="F83" t="n">
-        <v>1.0539</v>
+        <v>1.2817</v>
       </c>
     </row>
     <row r="84">
@@ -2271,19 +2271,19 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>6.76</v>
+        <v>6.65</v>
       </c>
       <c r="C84" t="n">
-        <v>676</v>
+        <v>665</v>
       </c>
       <c r="D84" t="n">
-        <v>0.0643</v>
+        <v>0.0519</v>
       </c>
       <c r="E84" t="n">
-        <v>0.1098</v>
+        <v>0.1151</v>
       </c>
       <c r="F84" t="n">
-        <v>0.4542</v>
+        <v>0.3251</v>
       </c>
     </row>
     <row r="85">
@@ -2293,19 +2293,19 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>13.78</v>
+        <v>14.94</v>
       </c>
       <c r="C85" t="n">
-        <v>1378</v>
+        <v>1494</v>
       </c>
       <c r="D85" t="n">
-        <v>0.0927</v>
+        <v>0.0921</v>
       </c>
       <c r="E85" t="n">
-        <v>0.1431</v>
+        <v>0.1374</v>
       </c>
       <c r="F85" t="n">
-        <v>0.5468</v>
+        <v>0.5648</v>
       </c>
     </row>
     <row r="86">
@@ -2315,19 +2315,19 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>5.03</v>
+        <v>4.69</v>
       </c>
       <c r="C86" t="n">
-        <v>503</v>
+        <v>469</v>
       </c>
       <c r="D86" t="n">
-        <v>0.0366</v>
+        <v>0.0193</v>
       </c>
       <c r="E86" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.0872</v>
       </c>
       <c r="F86" t="n">
-        <v>0.2607</v>
+        <v>0.0552</v>
       </c>
     </row>
     <row r="87">
@@ -2337,19 +2337,19 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>1.1</v>
+        <v>1.34</v>
       </c>
       <c r="C87" t="n">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="D87" t="n">
-        <v>-0.0769</v>
+        <v>-0.0265</v>
       </c>
       <c r="E87" t="n">
-        <v>0.2891</v>
+        <v>0.2928</v>
       </c>
       <c r="F87" t="n">
-        <v>-0.3161</v>
+        <v>-0.1399</v>
       </c>
     </row>
     <row r="88">
@@ -2359,19 +2359,19 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>1.45</v>
+        <v>1.29</v>
       </c>
       <c r="C88" t="n">
-        <v>145</v>
+        <v>129</v>
       </c>
       <c r="D88" t="n">
-        <v>0.0813</v>
+        <v>0.0568</v>
       </c>
       <c r="E88" t="n">
-        <v>0.204</v>
+        <v>0.2396</v>
       </c>
       <c r="F88" t="n">
-        <v>0.3279</v>
+        <v>0.1768</v>
       </c>
     </row>
     <row r="89">
@@ -2387,13 +2387,13 @@
         <v>108</v>
       </c>
       <c r="D89" t="n">
-        <v>0.3686</v>
+        <v>0.3079</v>
       </c>
       <c r="E89" t="n">
-        <v>0.5607</v>
+        <v>0.5248</v>
       </c>
       <c r="F89" t="n">
-        <v>0.6317</v>
+        <v>0.5592</v>
       </c>
     </row>
     <row r="90">
@@ -2403,19 +2403,19 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>4.16</v>
+        <v>3.02</v>
       </c>
       <c r="C90" t="n">
-        <v>416</v>
+        <v>302</v>
       </c>
       <c r="D90" t="n">
-        <v>0.06660000000000001</v>
+        <v>0.0001</v>
       </c>
       <c r="E90" t="n">
-        <v>0.1318</v>
+        <v>0.101</v>
       </c>
       <c r="F90" t="n">
-        <v>0.3954</v>
+        <v>-0.1422</v>
       </c>
     </row>
     <row r="91">
@@ -2425,19 +2425,19 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>24.5</v>
+        <v>31.08</v>
       </c>
       <c r="C91" t="n">
-        <v>2450</v>
+        <v>3108</v>
       </c>
       <c r="D91" t="n">
-        <v>0.1223</v>
+        <v>0.1472</v>
       </c>
       <c r="E91" t="n">
-        <v>0.1086</v>
+        <v>0.1224</v>
       </c>
       <c r="F91" t="n">
-        <v>0.9929</v>
+        <v>1.0851</v>
       </c>
     </row>
     <row r="92">
@@ -2447,19 +2447,19 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>2.98</v>
+        <v>3.16</v>
       </c>
       <c r="C92" t="n">
-        <v>298</v>
+        <v>316</v>
       </c>
       <c r="D92" t="n">
-        <v>-0.0834</v>
+        <v>-0.0586</v>
       </c>
       <c r="E92" t="n">
-        <v>0.0761</v>
+        <v>0.1016</v>
       </c>
       <c r="F92" t="n">
-        <v>-1.2855</v>
+        <v>-0.7185</v>
       </c>
     </row>
     <row r="93">
@@ -2469,19 +2469,19 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>4.12</v>
+        <v>4.01</v>
       </c>
       <c r="C93" t="n">
-        <v>412</v>
+        <v>401</v>
       </c>
       <c r="D93" t="n">
-        <v>-0.1114</v>
+        <v>-0.09520000000000001</v>
       </c>
       <c r="E93" t="n">
-        <v>0.1728</v>
+        <v>0.169</v>
       </c>
       <c r="F93" t="n">
-        <v>-0.7282999999999999</v>
+        <v>-0.6484</v>
       </c>
     </row>
     <row r="94">
@@ -2491,19 +2491,19 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>1.27</v>
+        <v>1.13</v>
       </c>
       <c r="C94" t="n">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="D94" t="n">
-        <v>0.0586</v>
+        <v>0.0239</v>
       </c>
       <c r="E94" t="n">
-        <v>0.3991</v>
+        <v>0.3271</v>
       </c>
       <c r="F94" t="n">
-        <v>0.1107</v>
+        <v>0.029</v>
       </c>
     </row>
     <row r="95">
@@ -2513,19 +2513,19 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>4.17</v>
+        <v>4.66</v>
       </c>
       <c r="C95" t="n">
-        <v>417</v>
+        <v>466</v>
       </c>
       <c r="D95" t="n">
-        <v>0.02</v>
+        <v>0.037</v>
       </c>
       <c r="E95" t="n">
-        <v>0.09180000000000001</v>
+        <v>0.1017</v>
       </c>
       <c r="F95" t="n">
-        <v>0.0606</v>
+        <v>0.2215</v>
       </c>
     </row>
     <row r="96">
@@ -2535,19 +2535,19 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>2.33</v>
+        <v>2.64</v>
       </c>
       <c r="C96" t="n">
-        <v>233</v>
+        <v>264</v>
       </c>
       <c r="D96" t="n">
-        <v>-0.095</v>
+        <v>-0.0578</v>
       </c>
       <c r="E96" t="n">
-        <v>0.3269</v>
+        <v>0.3032</v>
       </c>
       <c r="F96" t="n">
-        <v>-0.3347</v>
+        <v>-0.2383</v>
       </c>
     </row>
     <row r="97">
@@ -2557,19 +2557,19 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>3.45</v>
+        <v>2.67</v>
       </c>
       <c r="C97" t="n">
-        <v>345</v>
+        <v>267</v>
       </c>
       <c r="D97" t="n">
-        <v>0.5127</v>
+        <v>0.3882</v>
       </c>
       <c r="E97" t="n">
-        <v>0.5143</v>
+        <v>0.5476</v>
       </c>
       <c r="F97" t="n">
-        <v>0.9687</v>
+        <v>0.6826</v>
       </c>
     </row>
     <row r="98">
@@ -2579,19 +2579,19 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>4.82</v>
+        <v>4.42</v>
       </c>
       <c r="C98" t="n">
-        <v>482</v>
+        <v>442</v>
       </c>
       <c r="D98" t="n">
-        <v>0.644</v>
+        <v>0.5216</v>
       </c>
       <c r="E98" t="n">
-        <v>0.8361</v>
+        <v>0.8035</v>
       </c>
       <c r="F98" t="n">
-        <v>0.753</v>
+        <v>0.6312</v>
       </c>
     </row>
     <row r="99">
@@ -2601,19 +2601,19 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>1.02</v>
+        <v>0.96</v>
       </c>
       <c r="C99" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D99" t="n">
-        <v>0.0282</v>
+        <v>0.0121</v>
       </c>
       <c r="E99" t="n">
-        <v>0.2163</v>
+        <v>0.1839</v>
       </c>
       <c r="F99" t="n">
-        <v>0.06370000000000001</v>
+        <v>-0.013</v>
       </c>
     </row>
     <row r="100">
@@ -2623,19 +2623,19 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>11798.06</v>
+        <v>12265.96</v>
       </c>
       <c r="C100" t="n">
-        <v>1179806</v>
+        <v>1226596</v>
       </c>
       <c r="D100" t="n">
-        <v>0.0213</v>
+        <v>0.0247</v>
       </c>
       <c r="E100" t="n">
-        <v>0.0453</v>
+        <v>0.0498</v>
       </c>
       <c r="F100" t="n">
-        <v>0.1524</v>
+        <v>0.2058</v>
       </c>
     </row>
     <row r="101">
@@ -2645,19 +2645,19 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>1590.09</v>
+        <v>1642.33</v>
       </c>
       <c r="C101" t="n">
-        <v>159009</v>
+        <v>164233</v>
       </c>
       <c r="D101" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0129</v>
       </c>
       <c r="E101" t="n">
-        <v>0.0352</v>
+        <v>0.0381</v>
       </c>
       <c r="F101" t="n">
-        <v>-0.1606</v>
+        <v>-0.0395</v>
       </c>
     </row>
   </sheetData>

</xml_diff>